<commit_message>
feat: upgrade SEO metadata, custom animated icons, footer styling, and intake form validation
</commit_message>
<xml_diff>
--- a/public/contact_leads.xlsx
+++ b/public/contact_leads.xlsx
@@ -1,47 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Contact Leads" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Contact Leads" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Gmail / Insta Handle</t>
+  </si>
+  <si>
+    <t>Business / Company Name</t>
+  </si>
+  <si>
+    <t>Target Service Domain</t>
+  </si>
+  <si>
+    <t>Scope &amp; Budget</t>
+  </si>
+  <si>
+    <t>Project Objectives / Message</t>
+  </si>
+  <si>
+    <t>8/6/2026, 6:08:00 PM</t>
+  </si>
+  <si>
+    <t>Veloxa Demo Client</t>
+  </si>
+  <si>
+    <t>demo@veloxa.ai</t>
+  </si>
+  <si>
+    <t>Veloxa Systems Inc</t>
+  </si>
+  <si>
+    <t>AI Integration</t>
+  </si>
+  <si>
+    <t>₹15k - ₹20k</t>
+  </si>
+  <si>
+    <t>Automate customer intake workflows and custom AI integration.</t>
+  </si>
+  <si>
+    <t>8/7/2026, 12:43:31 AM</t>
+  </si>
+  <si>
+    <t>Test User</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>Acme Corp</t>
+  </si>
+  <si>
+    <t>₹5k - ₹10k</t>
+  </si>
+  <si>
+    <t>Hello world</t>
+  </si>
+  <si>
+    <t>8/8/2026, 1:32:52 AM</t>
+  </si>
+  <si>
+    <t>xzxz</t>
+  </si>
+  <si>
+    <t>@asas</t>
+  </si>
+  <si>
+    <t>dsdasas</t>
+  </si>
+  <si>
+    <t>saddas</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,11 +461,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="1" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
     <col min="4" max="4" width="28.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
@@ -408,78 +473,98 @@
     <col min="7" max="7" width="45.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Timestamp</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Full Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Gmail / Insta Handle</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Business / Company Name</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Target Service Domain</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Scope &amp; Budget</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Project Objectives / Message</v>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>8/6/2026, 6:08:00 PM</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Veloxa Demo Client</v>
-      </c>
-      <c r="C2" t="str">
-        <v>demo@veloxa.ai</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Veloxa Systems Inc</v>
-      </c>
-      <c r="E2" t="str">
-        <v>AI Integration</v>
-      </c>
-      <c r="F2" t="str">
-        <v>₹15k - ₹20k</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Automate customer intake workflows and custom AI integration.</v>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>8/7/2026, 12:43:31 AM</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Test User</v>
-      </c>
-      <c r="C3" t="str">
-        <v>test@gmail.com</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Acme Corp</v>
-      </c>
-      <c r="E3" t="str">
-        <v>AI Integration</v>
-      </c>
-      <c r="F3" t="str">
-        <v>₹5k - ₹10k</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Hello world</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: refine features timeline and frequency graph layout, enhance stepper UI, and enable intake validation
</commit_message>
<xml_diff>
--- a/public/contact_leads.xlsx
+++ b/public/contact_leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="35">
   <si>
     <t>Timestamp</t>
   </si>
@@ -86,6 +86,36 @@
   </si>
   <si>
     <t>saddas</t>
+  </si>
+  <si>
+    <t>8/21/2026, 4:14:38 AM</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>8/21/2026, 4:21:07 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 4:25:03 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 4:26:56 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 5:07:35 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 5:08:49 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 5:15:49 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 5:30:55 AM</t>
+  </si>
+  <si>
+    <t>8/21/2026, 5:55:02 PM</t>
   </si>
 </sst>
 </file>
@@ -462,8 +492,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr customHeight="1"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="22.83203125" customWidth="1"/>
     <col min="3" max="3" width="26.83203125" customWidth="1"/>
@@ -565,6 +595,213 @@
         <v>24</v>
       </c>
     </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): remove status bar, receipt container, input asterisks, and background star particles
</commit_message>
<xml_diff>
--- a/public/contact_leads.xlsx
+++ b/public/contact_leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="49">
   <si>
     <t>Timestamp</t>
   </si>
@@ -131,6 +131,33 @@
   </si>
   <si>
     <t>Need complete custom AI automated intake and CRM integration.</t>
+  </si>
+  <si>
+    <t>9/5/2026, 3:31:53 AM</t>
+  </si>
+  <si>
+    <t>kanhav sharma</t>
+  </si>
+  <si>
+    <t>wayneandtatecorp@gmail.com</t>
+  </si>
+  <si>
+    <t>IJK</t>
+  </si>
+  <si>
+    <t>Web Engineering</t>
+  </si>
+  <si>
+    <t>Negotiable Price</t>
+  </si>
+  <si>
+    <t>kjskdjsksjsjjas</t>
+  </si>
+  <si>
+    <t>9/5/2026, 3:32:32 AM</t>
+  </si>
+  <si>
+    <t>bbb</t>
   </si>
 </sst>
 </file>
@@ -510,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="22.83203125" customWidth="1"/>
@@ -843,6 +870,52 @@
         <v>39</v>
       </c>
     </row>
+    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "fix(ui): remove status bar, receipt container, input asterisks, and background star particles"
This reverts commit 044e903bcbc493cfc87cde1361828ef9429f1c5b.
</commit_message>
<xml_diff>
--- a/public/contact_leads.xlsx
+++ b/public/contact_leads.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="40">
   <si>
     <t>Timestamp</t>
   </si>
@@ -131,33 +131,6 @@
   </si>
   <si>
     <t>Need complete custom AI automated intake and CRM integration.</t>
-  </si>
-  <si>
-    <t>9/5/2026, 3:31:53 AM</t>
-  </si>
-  <si>
-    <t>kanhav sharma</t>
-  </si>
-  <si>
-    <t>wayneandtatecorp@gmail.com</t>
-  </si>
-  <si>
-    <t>IJK</t>
-  </si>
-  <si>
-    <t>Web Engineering</t>
-  </si>
-  <si>
-    <t>Negotiable Price</t>
-  </si>
-  <si>
-    <t>kjskdjsksjsjjas</t>
-  </si>
-  <si>
-    <t>9/5/2026, 3:32:32 AM</t>
-  </si>
-  <si>
-    <t>bbb</t>
   </si>
 </sst>
 </file>
@@ -537,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="22.83203125" customWidth="1"/>
@@ -870,52 +843,6 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>